<commit_message>
Module 6: ship the assembled report from a clean 1→2→3 run
Ran all three notebooks in order on TIP. The assembled report opens and
all 12 pages plus the FINAL link are functional — verified the fresh
report carries the corrected ../ relative links (7/7 resolve, one copy of
plotly.js).

Commits the regenerated outputs and report, adds ipc_rankings.xlsx (now
legitimately produced by notebook 2), and clears the .ipynb_checkpoints.
Notebooks are clean: sequential execution from 1, no error outputs, and
no leftover /home/jovyan paths or old output_* folder names in stored
output.

Module 6 is now reproducible end to end from a PATSTAT query and ready.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/6_patentreports/1_antibiotic_resistance/2_technology_network_output/technology_legend.xlsx
+++ b/6_patentreports/1_antibiotic_resistance/2_technology_network_output/technology_legend.xlsx
@@ -463,53 +463,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Antiinfective Therapy</t>
+          <t>Medical Technology</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A61P  31</t>
+          <t>A61K, A61K   8, A61K  33, A61K  35, A61K  36, A61K  41, A61K  48, A61P   1, A61P  11, A61P  13, A61P  15, A61P  17, A61P  29, A61P  35, A61P  37, A61Q  17, A61Q  19</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Antiinfective Therapeutics</t>
+          <t>Medical &amp; Pharmaceutical Technology</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1941</v>
+        <v>2106</v>
       </c>
       <c r="E2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9642857142857142</v>
+        <v>0.9285714285714285</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Medical Technology</t>
+          <t>Antiinfective Therapy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A61K, A61K   8, A61K  33, A61K  35, A61K  36, A61K  41, A61K  48, A61P   1, A61P  11, A61P  15, A61P  17, A61P  29, A61P  35, A61P  37, A61Q  19</t>
+          <t>A61P  31</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medical &amp; Pharmaceutical Technology</t>
+          <t>Antiinfective Therapeutics</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1860</v>
+        <v>2063</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9285714285714285</v>
+        <v>0.9642857142857142</v>
       </c>
     </row>
     <row r="4">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1385</v>
+        <v>1446</v>
       </c>
       <c r="E4" t="n">
         <v>27</v>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>960</v>
+        <v>993</v>
       </c>
       <c r="E5" t="n">
         <v>26</v>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>812</v>
+        <v>888</v>
       </c>
       <c r="E6" t="n">
         <v>26</v>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>768</v>
+        <v>801</v>
       </c>
       <c r="E7" t="n">
         <v>24</v>
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>709</v>
+        <v>753</v>
       </c>
       <c r="E8" t="n">
         <v>19</v>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>570</v>
+        <v>602</v>
       </c>
       <c r="E9" t="n">
         <v>24</v>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>516</v>
+        <v>546</v>
       </c>
       <c r="E10" t="n">
         <v>25</v>
@@ -697,53 +697,53 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chemistry (Heterocyclic)</t>
+          <t>Food Preservation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C07D 401, C07D 403, C07D 417, C07D 471, C07D 487, C07D 501</t>
+          <t>A23K  10, A23K  20, A23L   3, A23L  33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Antibiotic Chemistry - Heterocyclic</t>
+          <t>Food Preservation</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>452</v>
+        <v>472</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4642857142857142</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Food Preservation</t>
+          <t>Chemistry (Heterocyclic)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A23K  10, A23K  20, A23L   3, A23L  33</t>
+          <t>C07D 401, C07D 403, C07D 417, C07D 471, C07D 487, C07D 501</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Food Preservation</t>
+          <t>Antibiotic Chemistry - Heterocyclic</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E12" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.4642857142857142</v>
       </c>
     </row>
     <row r="13">
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>401</v>
+        <v>415</v>
       </c>
       <c r="E13" t="n">
         <v>23</v>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>361</v>
+        <v>392</v>
       </c>
       <c r="E14" t="n">
         <v>22</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>335</v>
+        <v>360</v>
       </c>
       <c r="E15" t="n">
         <v>23</v>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="E16" t="n">
         <v>23</v>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="E17" t="n">
         <v>23</v>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="E18" t="n">
         <v>23</v>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="E20" t="n">
         <v>10</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E21" t="n">
         <v>21</v>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E22" t="n">
         <v>21</v>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E23" t="n">
         <v>19</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E24" t="n">
         <v>20</v>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" t="n">
         <v>15</v>
@@ -1087,53 +1087,53 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Protein Production</t>
+          <t>Organic Chemistry</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C12P  21</t>
+          <t>C07F   5</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Protein Production</t>
+          <t>Organic Chemistry</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E26" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
-        <v>0.6071428571428571</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Organic Chemistry</t>
+          <t>Protein Production</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C07F   5</t>
+          <t>C12P  21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Organic Chemistry</t>
+          <t>Protein Production</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E27" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.6071428571428571</v>
       </c>
     </row>
     <row r="28">
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E28" t="n">
         <v>17</v>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E29" t="n">
         <v>9</v>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>

</xml_diff>